<commit_message>
Per-coach day comments (0009), strict initial+last names, roster-friendly importer
- day_comments table mirrors week_comments one level down: each coach's own
  attributed comment per athlete-day; the ✓ stays shared (locked 7). Legacy
  day_reviews comments migrate in 0009; the column is no longer written.
- Drill-in day cards: other coach's comment read-only above your own box.
  Athlete day card lists every coach's comment by name; green dots key off
  day_comments. Alert handled-state now counts a day comment as handling.
- shortName is now strictly first-initial + last name (B. McMahon) and is the
  single athlete-name format across the coach portal (grid, alerts, drill-in).
- Importer: a Goals row with name+email but blank mileage is a warned skip,
  not an error -- so the pre-filled roster template never blocks a posting.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/hooslog_week_plan_template.xlsx
+++ b/docs/templates/hooslog_week_plan_template.xlsx
@@ -1,19 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamhaydensheets/dev/hooslog/docs/templates/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5573630-08A5-5F46-BE3B-84998E00DDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="15980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Week Plan" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Goals" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="READ ME" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Week Plan" sheetId="1" r:id="rId1"/>
+    <sheet name="Goals" sheetId="2" r:id="rId2"/>
+    <sheet name="READ ME" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -22,102 +38,107 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t xml:space="preserve">HoosLog — Weekly Plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week of (Monday):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">← edit this one date; every day below updates itself</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WORKOUT PLAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR + hurdles + drills, WEIGHTS   (example — overwrite)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuesday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wednesday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thursday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saturday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sunday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow cells are yours: the Monday date and each day's plan. Leave a day blank for no plan. Don't add or delete rows.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATHLETE NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UVA EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WEEKLY GOAL (MILES)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One row per athlete. Email must be the athlete's UVA login email — it's how the upload matches people. Delete the example row before uploading.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example Athlete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abc1de@virginia.edu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HoosLog week-plan template — how it works</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Week Plan tab: set the Monday date (one yellow cell), type each day's plan in the yellow column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Goals tab: one row per athlete — name, UVA email, weekly mileage goal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Save, then drag this file into HoosLog (Coach → Upload week). Every athlete's week appears.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rules the upload depends on: don't rename tabs, don't add/delete rows or columns on the Week Plan tab,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">emails on the Goals tab must match athletes' HoosLog login emails, delete the example rows before upload.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recreated from the team's paper weekly sheet — same structure, same workflow. (docs/mockups/10)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+  <si>
+    <t>HoosLog — Weekly Plan</t>
+  </si>
+  <si>
+    <t>Week of (Monday):</t>
+  </si>
+  <si>
+    <t>← edit this one date; every day below updates itself</t>
+  </si>
+  <si>
+    <t>DAY</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>WORKOUT PLAN</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>TR + hurdles + drills, WEIGHTS   (example — overwrite)</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Yellow cells are yours: the Monday date and each day's plan. Leave a day blank for no plan. Don't add or delete rows.</t>
+  </si>
+  <si>
+    <t>ATHLETE NAME</t>
+  </si>
+  <si>
+    <t>UVA EMAIL</t>
+  </si>
+  <si>
+    <t>WEEKLY GOAL (MILES)</t>
+  </si>
+  <si>
+    <t>One row per athlete. Email must be the athlete's UVA login email — it's how the upload matches people. Delete the example row before uploading.</t>
+  </si>
+  <si>
+    <t>Example Athlete</t>
+  </si>
+  <si>
+    <t>abc1de@virginia.edu</t>
+  </si>
+  <si>
+    <t>HoosLog week-plan template — how it works</t>
+  </si>
+  <si>
+    <t>1. Week Plan tab: set the Monday date (one yellow cell), type each day's plan in the yellow column.</t>
+  </si>
+  <si>
+    <t>2. Goals tab: one row per athlete — name, UVA email, weekly mileage goal.</t>
+  </si>
+  <si>
+    <t>3. Save, then drag this file into HoosLog (Coach → Upload week). Every athlete's week appears.</t>
+  </si>
+  <si>
+    <t>Rules the upload depends on: don't rename tabs, don't add/delete rows or columns on the Week Plan tab,</t>
+  </si>
+  <si>
+    <t>emails on the Goals tab must match athletes' HoosLog login emails, delete the example rows before upload.</t>
+  </si>
+  <si>
+    <t>Recreated from the team's paper weekly sheet — same structure, same workflow. (docs/mockups/10)</t>
+  </si>
+  <si>
+    <t>William Sheets</t>
+  </si>
+  <si>
+    <t>fnh4mv@virginia.edu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-    <numFmt numFmtId="166" formatCode="ddd\ m/d"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -128,62 +149,54 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF232D4B"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF232D4B"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FF232D4B"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF232D4B"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <color rgb="FF5C6478"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="10"/>
       <color rgb="FF5C6478"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -208,14 +221,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFE6E8EE"/>
       </left>
@@ -231,97 +244,40 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="14">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -380,47 +336,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF232D4B"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -428,12 +400,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -462,7 +434,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -483,7 +455,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -534,7 +506,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -552,43 +524,42 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="64"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:3" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>46244</v>
+      <c r="B3" s="3">
+        <v>46258</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -599,109 +570,101 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <f aca="false">$B$3</f>
-        <v>46244</v>
+      <c r="B6" s="7">
+        <f>$B$3</f>
+        <v>46258</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7" t="n">
-        <f aca="false">$B$3+1</f>
-        <v>46245</v>
+      <c r="B7" s="7">
+        <f>$B$3+1</f>
+        <v>46259</v>
       </c>
       <c r="C7" s="9"/>
     </row>
-    <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="7" t="n">
-        <f aca="false">$B$3+2</f>
-        <v>46246</v>
+      <c r="B8" s="7">
+        <f>$B$3+2</f>
+        <v>46260</v>
       </c>
       <c r="C8" s="9"/>
     </row>
-    <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7" t="n">
-        <f aca="false">$B$3+3</f>
-        <v>46247</v>
+      <c r="B9" s="7">
+        <f>$B$3+3</f>
+        <v>46261</v>
       </c>
       <c r="C9" s="9"/>
     </row>
-    <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <f aca="false">$B$3+4</f>
-        <v>46248</v>
+      <c r="B10" s="7">
+        <f>$B$3+4</f>
+        <v>46262</v>
       </c>
       <c r="C10" s="9"/>
     </row>
-    <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <f aca="false">$B$3+5</f>
-        <v>46249</v>
+      <c r="B11" s="7">
+        <f>$B$3+5</f>
+        <v>46263</v>
       </c>
       <c r="C11" s="9"/>
     </row>
-    <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <f aca="false">$B$3+6</f>
-        <v>46250</v>
+      <c r="B12" s="7">
+        <f>$B$3+6</f>
+        <v>46264</v>
       </c>
       <c r="C12" s="9"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:5" ht="39" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -715,217 +678,213 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="11" t="n">
+      <c r="C2" s="11">
         <v>70</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="12">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12"/>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12"/>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="12"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="12"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="12"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="12"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="12"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="12"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="12"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="12"/>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="12"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="12"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="12"/>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="12"/>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="12"/>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="12"/>
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{3CF7B516-972C-A44D-B248-1C013AFE1E09}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
+    <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="13"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="13"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Importer: mileage ranges parse to their midpoint; date-converted ranges get a plain fix
- '45-49', '45 – 49', '45 to 49' all read as 47 with a preview note naming
  the conversion; backwards ranges error with the corrected order.
- A goal cell Excel silently turned into a date (typing '5-10' does this)
  errors with the fix ('type it as 5 to 10, or format the cell as Text')
  instead of parsing as nonsense.
- Blank goals were already warned skips (unchanged, covered by the new
  scripts/test-goal-parsing.ts harness + fixtures).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/hooslog_week_plan_template.xlsx
+++ b/docs/templates/hooslog_week_plan_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamhaydensheets/dev/hooslog/docs/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5573630-08A5-5F46-BE3B-84998E00DDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A4F384-A722-064C-81D7-2CB2FFFC9CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="15980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,9 +61,6 @@
     <t>Monday</t>
   </si>
   <si>
-    <t>TR + hurdles + drills, WEIGHTS   (example — overwrite)</t>
-  </si>
-  <si>
     <t>Tuesday</t>
   </si>
   <si>
@@ -128,6 +125,9 @@
   </si>
   <si>
     <t>fnh4mv@virginia.edu</t>
+  </si>
+  <si>
+    <t>TR + hurdles + drills, WEIGHTS   (</t>
   </si>
 </sst>
 </file>
@@ -579,12 +579,12 @@
         <v>46258</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" s="7">
         <f>$B$3+1</f>
@@ -594,7 +594,7 @@
     </row>
     <row r="8" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="7">
         <f>$B$3+2</f>
@@ -604,7 +604,7 @@
     </row>
     <row r="9" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="7">
         <f>$B$3+3</f>
@@ -614,7 +614,7 @@
     </row>
     <row r="10" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="7">
         <f>$B$3+4</f>
@@ -624,7 +624,7 @@
     </row>
     <row r="11" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="7">
         <f>$B$3+5</f>
@@ -634,7 +634,7 @@
     </row>
     <row r="12" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="7">
         <f>$B$3+6</f>
@@ -644,7 +644,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -666,24 +666,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="39" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="10" t="s">
         <v>17</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>19</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>20</v>
       </c>
       <c r="C2" s="11">
         <v>70</v>
@@ -691,10 +691,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>28</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>29</v>
       </c>
       <c r="C3" s="12">
         <v>58</v>
@@ -844,7 +844,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
@@ -852,17 +852,17 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -870,17 +870,17 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>